<commit_message>
Update mean daily temperature for loop
</commit_message>
<xml_diff>
--- a/00_Data/Datasets_metadata.xlsx
+++ b/00_Data/Datasets_metadata.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felicitycharles/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felicitycharles/Desktop/GitHub/Fire_freq_pred_modelling/00_Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCC7F1FA-A4A7-324A-8ABD-036C07783D00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCBAF504-660F-FC4F-AD7B-3166D87CEF29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="940" yWindow="1020" windowWidth="28800" windowHeight="15380" xr2:uid="{CFB87D9E-A38C-4243-925E-2D890E6206AE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="90">
   <si>
     <t>Dataset</t>
   </si>
@@ -1161,6 +1161,9 @@
       <c r="A18" s="3" t="s">
         <v>53</v>
       </c>
+      <c r="B18" t="s">
+        <v>9</v>
+      </c>
       <c r="C18">
         <v>2021</v>
       </c>
@@ -1184,6 +1187,9 @@
       <c r="A19" s="3" t="s">
         <v>87</v>
       </c>
+      <c r="B19" t="s">
+        <v>9</v>
+      </c>
       <c r="C19">
         <v>2022</v>
       </c>
@@ -1206,6 +1212,9 @@
     <row r="20" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
         <v>88</v>
+      </c>
+      <c r="B20" t="s">
+        <v>9</v>
       </c>
       <c r="C20">
         <v>2023</v>

</xml_diff>